<commit_message>
Step 1: simple_list helper + 7 new non-table scrapers (전북/전남)
Add scrapers/_helpers/simple_list.py — scrapes pages that have article
links but no <table> (list.jinan, list.jangsu, list.gochang, boardList.do,
index.9is portal pages). Key fix: uses r.text not r.content; lxml fails
to detect encoding from bytes on some Korean sites.

New scrapers (7 new T entries, 182→189 T, 192→185 F):
  진안군 공지사항 (list.jinan / BBS_0000026)
  장수군 공지사항 (list.jangsu / BBS_0000003)
  고창군 공지사항 + 고시공고 (list.gochang / BBS_0000083, BBS_0000180)
  고흥군 공지사항 (boardList.do/boardView.do)
  함평군 공지사항 (boardList.do/boardView.do)
  완주군 고시공고 (index.9is portal, jeonbuk_batch)
  임실군 고시공고 (list.imsil / BBS_0000003, jeonbuk_batch)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/links_v2.xlsx
+++ b/links_v2.xlsx
@@ -15759,7 +15759,7 @@
       </c>
       <c r="F201" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -15789,7 +15789,7 @@
       </c>
       <c r="F202" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -15909,7 +15909,7 @@
       </c>
       <c r="F206" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -16089,7 +16089,7 @@
       </c>
       <c r="F212" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -16119,7 +16119,7 @@
       </c>
       <c r="F213" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -16689,7 +16689,7 @@
       </c>
       <c r="F232" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17169,7 +17169,7 @@
       </c>
       <c r="F248" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 1 complete: 315T scrapers + UI overhaul (dark sidebar, search, live feed)
Scrapers (315T / 59F):
- Add Playwright boardlist.do scrapers for 경북/경남개발공사 (gongsa_web_batch)
- Add saeol.py helper + portal_bbs/board/fn_articleLink adapters
- Add playwright_web.py for .web CMS sites (경남, 강원)
- Add gyeongnam_web_batch, gangwon_web_batch, chungbuk_web_batch
- Add gwangju_si, ddc (대전도시공사)
- Refactor _sangju_tc helper; add 상주시 공지사항 scraper
- Expand gyeonggi, jeonbuk, jeonnam, busan, chungnam, sejong batches
- Update links_v2.xlsx classification (315T)

UI:
- Dark navy sidebar matching header, with live search/filter
- RecentFeed: landing page shows 24 most-recent notices from all regions
- Animated skeleton loading cards replacing plain "불러오는 중…" text
- Notice count badge in section header after Supabase load
- Relative date formatting (오늘/어제/N일 전)
- Fix NoticePlaceholder: remove stale "크롤러 미연결" message

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/links_v2.xlsx
+++ b/links_v2.xlsx
@@ -9879,7 +9879,7 @@
       </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -9909,7 +9909,7 @@
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -9939,7 +9939,7 @@
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -9999,7 +9999,7 @@
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -10179,7 +10179,7 @@
       </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -10269,7 +10269,7 @@
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -10479,7 +10479,7 @@
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -10509,7 +10509,7 @@
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -10779,7 +10779,7 @@
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -11169,7 +11169,7 @@
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -11199,7 +11199,7 @@
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -11319,7 +11319,7 @@
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -11619,7 +11619,7 @@
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -11649,7 +11649,7 @@
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -11679,7 +11679,7 @@
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -11739,7 +11739,7 @@
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -11769,7 +11769,7 @@
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -11799,7 +11799,7 @@
       </c>
       <c r="F69" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -11829,7 +11829,7 @@
       </c>
       <c r="F70" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -11889,7 +11889,7 @@
       </c>
       <c r="F72" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -11919,7 +11919,7 @@
       </c>
       <c r="F73" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -11949,7 +11949,7 @@
       </c>
       <c r="F74" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -12099,7 +12099,7 @@
       </c>
       <c r="F79" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -12249,7 +12249,7 @@
       </c>
       <c r="F84" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -12309,7 +12309,7 @@
       </c>
       <c r="F86" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -12339,7 +12339,7 @@
       </c>
       <c r="F87" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -12489,7 +12489,7 @@
       </c>
       <c r="F92" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -12549,7 +12549,7 @@
       </c>
       <c r="F94" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -12609,7 +12609,7 @@
       </c>
       <c r="F96" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -12699,7 +12699,7 @@
       </c>
       <c r="F99" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -12759,7 +12759,7 @@
       </c>
       <c r="F101" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -12849,7 +12849,7 @@
       </c>
       <c r="F104" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -13089,7 +13089,7 @@
       </c>
       <c r="F112" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -13239,7 +13239,7 @@
       </c>
       <c r="F117" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -13269,7 +13269,7 @@
       </c>
       <c r="F118" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -13419,7 +13419,7 @@
       </c>
       <c r="F123" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -13539,7 +13539,7 @@
       </c>
       <c r="F127" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -13659,7 +13659,7 @@
       </c>
       <c r="F131" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -13869,7 +13869,7 @@
       </c>
       <c r="F138" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -13899,7 +13899,7 @@
       </c>
       <c r="F139" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -13929,7 +13929,7 @@
       </c>
       <c r="F140" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -13959,7 +13959,7 @@
       </c>
       <c r="F141" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -14019,7 +14019,7 @@
       </c>
       <c r="F143" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -14049,7 +14049,7 @@
       </c>
       <c r="F144" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -14079,7 +14079,7 @@
       </c>
       <c r="F145" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -15069,7 +15069,7 @@
       </c>
       <c r="F178" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -15099,7 +15099,7 @@
       </c>
       <c r="F179" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -15999,7 +15999,7 @@
       </c>
       <c r="F209" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -16359,7 +16359,7 @@
       </c>
       <c r="F221" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -16599,7 +16599,7 @@
       </c>
       <c r="F229" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -16659,7 +16659,7 @@
       </c>
       <c r="F231" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17019,7 +17019,7 @@
       </c>
       <c r="F243" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17079,7 +17079,7 @@
       </c>
       <c r="F245" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17199,7 +17199,7 @@
       </c>
       <c r="F249" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17499,7 +17499,7 @@
       </c>
       <c r="F259" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17529,7 +17529,7 @@
       </c>
       <c r="F260" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17559,7 +17559,7 @@
       </c>
       <c r="F261" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17589,7 +17589,7 @@
       </c>
       <c r="F262" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17619,7 +17619,7 @@
       </c>
       <c r="F263" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17709,7 +17709,7 @@
       </c>
       <c r="F266" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17739,7 +17739,7 @@
       </c>
       <c r="F267" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17769,7 +17769,7 @@
       </c>
       <c r="F268" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17799,7 +17799,7 @@
       </c>
       <c r="F269" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17829,7 +17829,7 @@
       </c>
       <c r="F270" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17859,7 +17859,7 @@
       </c>
       <c r="F271" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17889,7 +17889,7 @@
       </c>
       <c r="F272" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17919,7 +17919,7 @@
       </c>
       <c r="F273" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17949,7 +17949,7 @@
       </c>
       <c r="F274" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -17979,7 +17979,7 @@
       </c>
       <c r="F275" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18009,7 +18009,7 @@
       </c>
       <c r="F276" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18039,7 +18039,7 @@
       </c>
       <c r="F277" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18069,7 +18069,7 @@
       </c>
       <c r="F278" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18099,7 +18099,7 @@
       </c>
       <c r="F279" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18129,7 +18129,7 @@
       </c>
       <c r="F280" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18159,7 +18159,7 @@
       </c>
       <c r="F281" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18189,7 +18189,7 @@
       </c>
       <c r="F282" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18219,7 +18219,7 @@
       </c>
       <c r="F283" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18249,7 +18249,7 @@
       </c>
       <c r="F284" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18279,7 +18279,7 @@
       </c>
       <c r="F285" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18429,7 +18429,7 @@
       </c>
       <c r="F290" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18459,7 +18459,7 @@
       </c>
       <c r="F291" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18489,7 +18489,7 @@
       </c>
       <c r="F292" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18519,7 +18519,7 @@
       </c>
       <c r="F293" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18549,7 +18549,7 @@
       </c>
       <c r="F294" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18579,7 +18579,7 @@
       </c>
       <c r="F295" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18609,7 +18609,7 @@
       </c>
       <c r="F296" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18639,7 +18639,7 @@
       </c>
       <c r="F297" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18729,7 +18729,7 @@
       </c>
       <c r="F300" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18759,7 +18759,7 @@
       </c>
       <c r="F301" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18849,7 +18849,7 @@
       </c>
       <c r="F304" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18879,7 +18879,7 @@
       </c>
       <c r="F305" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18909,7 +18909,7 @@
       </c>
       <c r="F306" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18939,7 +18939,7 @@
       </c>
       <c r="F307" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18969,7 +18969,7 @@
       </c>
       <c r="F308" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -18999,7 +18999,7 @@
       </c>
       <c r="F309" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19029,7 +19029,7 @@
       </c>
       <c r="F310" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19059,7 +19059,7 @@
       </c>
       <c r="F311" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19149,7 +19149,7 @@
       </c>
       <c r="F314" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19179,7 +19179,7 @@
       </c>
       <c r="F315" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19209,7 +19209,7 @@
       </c>
       <c r="F316" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19239,7 +19239,7 @@
       </c>
       <c r="F317" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19299,7 +19299,7 @@
       </c>
       <c r="F319" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19389,7 +19389,7 @@
       </c>
       <c r="F322" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19419,7 +19419,7 @@
       </c>
       <c r="F323" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19449,7 +19449,7 @@
       </c>
       <c r="F324" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19479,7 +19479,7 @@
       </c>
       <c r="F325" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19569,7 +19569,7 @@
       </c>
       <c r="F328" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19599,7 +19599,7 @@
       </c>
       <c r="F329" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19629,7 +19629,7 @@
       </c>
       <c r="F330" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19659,7 +19659,7 @@
       </c>
       <c r="F331" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19749,7 +19749,7 @@
       </c>
       <c r="F334" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19809,7 +19809,7 @@
       </c>
       <c r="F336" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19839,7 +19839,7 @@
       </c>
       <c r="F337" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19869,7 +19869,7 @@
       </c>
       <c r="F338" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -19899,7 +19899,7 @@
       </c>
       <c r="F339" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -20079,7 +20079,7 @@
       </c>
       <c r="F345" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -20289,7 +20289,7 @@
       </c>
       <c r="F352" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -20469,7 +20469,7 @@
       </c>
       <c r="F358" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -20499,7 +20499,7 @@
       </c>
       <c r="F359" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -20589,7 +20589,7 @@
       </c>
       <c r="F362" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -20619,7 +20619,7 @@
       </c>
       <c r="F363" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -20709,7 +20709,7 @@
       </c>
       <c r="F366" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -20739,7 +20739,7 @@
       </c>
       <c r="F367" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -20829,7 +20829,7 @@
       </c>
       <c r="F370" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -20859,7 +20859,7 @@
       </c>
       <c r="F371" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -20949,7 +20949,7 @@
       </c>
       <c r="F374" s="0" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
     </row>

</xml_diff>